<commit_message>
Add Token Usage by Size tab: quarterly avg monthly tokens per company by segment
Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Blended_Token_Pricing_Frontier_and_Open_Weight_Models.xlsx
+++ b/Blended_Token_Pricing_Frontier_and_Open_Weight_Models.xlsx
@@ -11,8 +11,9 @@
     <sheet name="Price History" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Current Snapshot" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Quarterly Series" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Charts" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Sources" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Token Usage by Size" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Charts" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Sources" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Price History'!$A$1:$N$158</definedName>
@@ -24,11 +25,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00###"/>
+    <numFmt numFmtId="166" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -57,6 +59,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00C00000"/>
     </font>
   </fonts>
   <fills count="7">
@@ -104,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -132,6 +138,12 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -210,6 +222,297 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="12"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Avg monthly tokens per company by size (millions, log scale)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Token Usage by Size'!B4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="5"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Token Usage by Size'!$A$5:$A$19</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Token Usage by Size'!$B$5:$B$19</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Token Usage by Size'!C4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="5"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Token Usage by Size'!$A$5:$A$19</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Token Usage by Size'!$C$5:$C$19</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Token Usage by Size'!D4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="5"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Token Usage by Size'!$A$5:$A$19</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Token Usage by Size'!$D$5:$D$19</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'Token Usage by Size'!E4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="5"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Token Usage by Size'!$A$5:$A$19</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Token Usage by Size'!$E$5:$E$19</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <tx>
+            <strRef>
+              <f>'Token Usage by Size'!F4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="5"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Token Usage by Size'!$A$5:$A$19</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Token Usage by Size'!$F$5:$F$19</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="5"/>
+          <order val="5"/>
+          <tx>
+            <strRef>
+              <f>'Token Usage by Size'!G4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="5"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Token Usage by Size'!$A$5:$A$19</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Token Usage by Size'!$G$5:$G$19</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Quarter</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <logBase val="10"/>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Millions of tokens per company per month</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="12"/>
   <chart>
@@ -432,7 +735,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="12"/>
   <chart>
@@ -723,7 +1026,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="12"/>
   <chart>
@@ -913,6 +1216,33 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="9360000" cy="4320000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -1272,7 +1602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B33"/>
+  <dimension ref="B1:B34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1382,109 +1712,116 @@
     <row r="17" ht="30" customHeight="1">
       <c r="B17" s="2" t="inlineStr">
         <is>
+          <t>- Token Usage by Size: quarterly time series of estimated average monthly token consumption per company, by company-size segment (modeled estimates calibrated to Ramp AI Index, Deloitte, OpenAI Enterprise Signals, and VendorBenchmark anchors; methodology on the sheet).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="B18" s="2" t="inlineStr">
+        <is>
           <t>- Charts: blended price trajectories on a log scale - frontier flagships, open-weight flagships, and budget tiers.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="2" t="inlineStr">
+    <row r="19">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>- Sources: pricing pages, launch announcements, and trackers used.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="B19" s="2" t="inlineStr"/>
-    </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="B20" s="3" t="inlineStr">
+    <row r="20">
+      <c r="B20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Methodology notes &amp; caveats</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>1. Prices are standard pay-as-you-go list rates for the base (short) context tier. Long-context surcharges, cached-input rates, batch (-50%), priority/fast modes, and free tiers are excluded (noted where material).</t>
         </is>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>2. Reasoning models bill hidden reasoning tokens at the output rate; the blended figure understates their effective cost per visible token.</t>
+          <t>1. Prices are standard pay-as-you-go list rates for the base (short) context tier. Long-context surcharges, cached-input rates, batch (-50%), priority/fast modes, and free tiers are excluded (noted where material).</t>
         </is>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>3. Chinese CNY list prices converted at the rates published by the trackers used (~6.75-7.1 CNY/USD); conversion noted in the Basis column.</t>
+          <t>2. Reasoning models bill hidden reasoning tokens at the output rate; the blended figure understates their effective cost per visible token.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>4. Date precision: 'approx' marks launch dates estimated to the month from secondary sources; 'exact' dates come from vendor announcements.</t>
+          <t>3. Chinese CNY list prices converted at the rates published by the trackers used (~6.75-7.1 CNY/USD); conversion noted in the Basis column.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>5. Promotional prices are recorded as events and flagged (e.g. GPT-5.6 Sol's $4/$20 promo through Nov 2026; DeepSeek's off-peak windows).</t>
+          <t>4. Date precision: 'approx' marks launch dates estimated to the month from secondary sources; 'exact' dates come from vendor announcements.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>6. Open-weight hosted rates vary 2-4x across hosts; the Basis column names the reference host. Third-party host rates for the same model differ from the first-party rate shown.</t>
+          <t>5. Promotional prices are recorded as events and flagged (e.g. GPT-5.6 Sol's $4/$20 promo through Nov 2026; DeepSeek's off-peak windows).</t>
         </is>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="B27" s="2" t="inlineStr">
         <is>
+          <t>6. Open-weight hosted rates vary 2-4x across hosts; the Basis column names the reference host. Third-party host rates for the same model differ from the first-party rate shown.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="B28" s="2" t="inlineStr">
+        <is>
           <t>7. Tokenizers differ across vendors (e.g. Claude Sonnet 5 produces ~30% more tokens for the same text), so $/token is not a perfect cross-vendor unit of work.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="B28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="B29" s="3" t="inlineStr">
+    <row r="29">
+      <c r="B29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>Headline findings</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="30" customHeight="1">
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>- Frontier flagship blended price fell from $37.50 (GPT-4, Mar 2023) to a floor of ~$3.44 (GPT-5, Aug 2025), then REBOUNDED to $8-11+ in 2026 as reasoning-heavy flagships (GPT-5.5/5.6 at $5/$30, Claude Fable 5 at $10/$50) reset the ceiling.</t>
         </is>
       </c>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>- The budget tier collapsed &gt;99%: $2.00 blended (GPT-3.5 Turbo, Mar 2023) to $0.20-0.45 (GPT-5.6 Luna, Gemini Flash-Lite class, 2026).</t>
+          <t>- Frontier flagship blended price fell from $37.50 (GPT-4, Mar 2023) to a floor of ~$3.44 (GPT-5, Aug 2025), then REBOUNDED to $8-11+ in 2026 as reasoning-heavy flagships (GPT-5.5/5.6 at $5/$30, Claude Fable 5 at $10/$50) reset the ceiling.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>- Open-weight flagships remain 3-10x cheaper than closed flagships, but their launch prices are rising (Kimi K3 at $6.00 blended is the most expensive open-weight launch to date).</t>
+          <t>- The budget tier collapsed &gt;99%: $2.00 blended (GPT-3.5 Turbo, Mar 2023) to $0.20-0.45 (GPT-5.6 Luna, Gemini Flash-Lite class, 2026).</t>
         </is>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>- Open-weight flagships remain 3-10x cheaper than closed flagships, but their launch prices are rising (Kimi K3 at $6.00 blended is the most expensive open-weight launch to date).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>- China's open-weight labs (DeepSeek, Qwen, Kimi, GLM) anchor the global price floor; DeepSeek V4 Flash off-peak reaches $0.33 blended.</t>
         </is>
@@ -19546,17 +19883,512 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B74:B74"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
-    <row r="74">
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>Y axes are logarithmic. Gaps before a lineage's first launch are blank. Source: Quarterly Series sheet.</t>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Estimated average monthly LLM token consumption per company, by company size - millions of tokens per company per month</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t>MODELED ESTIMATES calibrated to published anchors (see notes below) - not vendor-reported data. Includes API and subscription-mediated usage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="42" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Quarter</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Small business (1-99 emp.)</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Mid-market (100-999 emp.)</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Enterprise (1,000-9,999 emp.)</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Large enterprise (10,000+ emp.)</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>AI-native startup (memo)</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>All companies - median (memo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>2023 Q1</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="18" t="n">
+        <v>15</v>
+      </c>
+      <c r="D5" s="18" t="n">
+        <v>90</v>
+      </c>
+      <c r="E5" s="18" t="n">
+        <v>500</v>
+      </c>
+      <c r="F5" s="18" t="n">
+        <v>60</v>
+      </c>
+      <c r="G5" s="17" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>2023 Q2</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C6" s="18" t="n">
+        <v>22</v>
+      </c>
+      <c r="D6" s="18" t="n">
+        <v>140</v>
+      </c>
+      <c r="E6" s="18" t="n">
+        <v>800</v>
+      </c>
+      <c r="F6" s="18" t="n">
+        <v>120</v>
+      </c>
+      <c r="G6" s="17" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>2023 Q3</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="C7" s="18" t="n">
+        <v>32</v>
+      </c>
+      <c r="D7" s="18" t="n">
+        <v>210</v>
+      </c>
+      <c r="E7" s="18" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F7" s="18" t="n">
+        <v>230</v>
+      </c>
+      <c r="G7" s="17" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>2023 Q4</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="C8" s="18" t="n">
+        <v>48</v>
+      </c>
+      <c r="D8" s="18" t="n">
+        <v>320</v>
+      </c>
+      <c r="E8" s="18" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F8" s="18" t="n">
+        <v>420</v>
+      </c>
+      <c r="G8" s="17" t="n">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>2024 Q1</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="C9" s="18" t="n">
+        <v>70</v>
+      </c>
+      <c r="D9" s="18" t="n">
+        <v>480</v>
+      </c>
+      <c r="E9" s="18" t="n">
+        <v>3100</v>
+      </c>
+      <c r="F9" s="18" t="n">
+        <v>750</v>
+      </c>
+      <c r="G9" s="17" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>2024 Q2</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="C10" s="18" t="n">
+        <v>100</v>
+      </c>
+      <c r="D10" s="18" t="n">
+        <v>720</v>
+      </c>
+      <c r="E10" s="18" t="n">
+        <v>4800</v>
+      </c>
+      <c r="F10" s="18" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G10" s="18" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>2024 Q3</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="C11" s="18" t="n">
+        <v>145</v>
+      </c>
+      <c r="D11" s="18" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E11" s="18" t="n">
+        <v>7200</v>
+      </c>
+      <c r="F11" s="18" t="n">
+        <v>2200</v>
+      </c>
+      <c r="G11" s="18" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>2024 Q4</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="n">
+        <v>13</v>
+      </c>
+      <c r="C12" s="18" t="n">
+        <v>210</v>
+      </c>
+      <c r="D12" s="18" t="n">
+        <v>1600</v>
+      </c>
+      <c r="E12" s="18" t="n">
+        <v>11000</v>
+      </c>
+      <c r="F12" s="18" t="n">
+        <v>3700</v>
+      </c>
+      <c r="G12" s="18" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>2025 Q1</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="n">
+        <v>18</v>
+      </c>
+      <c r="C13" s="18" t="n">
+        <v>300</v>
+      </c>
+      <c r="D13" s="18" t="n">
+        <v>2400</v>
+      </c>
+      <c r="E13" s="18" t="n">
+        <v>17000</v>
+      </c>
+      <c r="F13" s="18" t="n">
+        <v>6000</v>
+      </c>
+      <c r="G13" s="18" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>2025 Q2</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="n">
+        <v>28</v>
+      </c>
+      <c r="C14" s="18" t="n">
+        <v>470</v>
+      </c>
+      <c r="D14" s="18" t="n">
+        <v>3800</v>
+      </c>
+      <c r="E14" s="18" t="n">
+        <v>27000</v>
+      </c>
+      <c r="F14" s="18" t="n">
+        <v>10000</v>
+      </c>
+      <c r="G14" s="18" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t>2025 Q3</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="n">
+        <v>45</v>
+      </c>
+      <c r="C15" s="18" t="n">
+        <v>750</v>
+      </c>
+      <c r="D15" s="18" t="n">
+        <v>6200</v>
+      </c>
+      <c r="E15" s="18" t="n">
+        <v>44000</v>
+      </c>
+      <c r="F15" s="18" t="n">
+        <v>16500</v>
+      </c>
+      <c r="G15" s="18" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>2025 Q4</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="n">
+        <v>75</v>
+      </c>
+      <c r="C16" s="18" t="n">
+        <v>1250</v>
+      </c>
+      <c r="D16" s="18" t="n">
+        <v>10500</v>
+      </c>
+      <c r="E16" s="18" t="n">
+        <v>74000</v>
+      </c>
+      <c r="F16" s="18" t="n">
+        <v>27000</v>
+      </c>
+      <c r="G16" s="18" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>2026 Q1</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="n">
+        <v>130</v>
+      </c>
+      <c r="C17" s="18" t="n">
+        <v>2150</v>
+      </c>
+      <c r="D17" s="18" t="n">
+        <v>18000</v>
+      </c>
+      <c r="E17" s="18" t="n">
+        <v>128000</v>
+      </c>
+      <c r="F17" s="18" t="n">
+        <v>44000</v>
+      </c>
+      <c r="G17" s="18" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>2026 Q2</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="n">
+        <v>200</v>
+      </c>
+      <c r="C18" s="18" t="n">
+        <v>3300</v>
+      </c>
+      <c r="D18" s="18" t="n">
+        <v>28000</v>
+      </c>
+      <c r="E18" s="18" t="n">
+        <v>200000</v>
+      </c>
+      <c r="F18" s="18" t="n">
+        <v>68000</v>
+      </c>
+      <c r="G18" s="18" t="n">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>2026 Q3</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="n">
+        <v>280</v>
+      </c>
+      <c r="C19" s="18" t="n">
+        <v>4600</v>
+      </c>
+      <c r="D19" s="18" t="n">
+        <v>39000</v>
+      </c>
+      <c r="E19" s="18" t="n">
+        <v>280000</v>
+      </c>
+      <c r="F19" s="18" t="n">
+        <v>95000</v>
+      </c>
+      <c r="G19" s="18" t="n">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1">
+      <c r="A21" s="19" t="inlineStr">
+        <is>
+          <t>How this series was built:</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="45" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>1. Anchor (2026 Q2): Ramp AI Index (Apr-Jun 2026, 70,000+ US businesses) - median company token spend $2,246/month at an observed effective rate of $0.72 per 1M tokens implies ~3.1B tokens/month for the median Ramp-tracked (mid-market, tech-forward) company; average spend $140,842/month implies ~200B tokens for the large-enterprise average.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="45" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>2. Growth path: Ramp reports token usage among businesses with connected AI grew 1,001% (~11x) from Jan 2025 to Apr 2026; each segment's series is backcast at that pace for 2025-2026 and at slower adoption-era rates for 2023-2024 (ChatGPT API launched Mar 2023).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="45" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>3. Cross-checks: Deloitte 2026 (cited by OpenRouter): 67% of enterprises consume &gt;1B tokens/month - consistent with the Enterprise column crossing 1B in 2024 and reaching ~28-39B in 2026. VendorBenchmark 2026: enterprise LLM API spend of $4-22 per employee/month supports the Enterprise and Large-enterprise levels. OpenAI Enterprise Signals (Jun 2026): top-decile 'frontier firms' generate 8.3x the output tokens per active user of typical firms - reflected in the AI-native startup memo column.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="45" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>4. Segment averages are means; token usage is power-law distributed within every segment (Ramp: median $2,246 vs average $140,842 monthly spend), so a segment's typical company sits well below its average. The 'All companies - median' memo column is the better 'typical firm' line.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="45" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>5. Usage includes tokens consumed through subscription products (ChatGPT/Claude/Copilot seats) valued at effective token rates, not only direct API billing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="45" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Caveats: no vendor publishes tokens-by-company-size; treat levels as order-of-magnitude estimates. Growth rates and 2026 anchors are well-sourced; 2023-2024 levels are extrapolations. Aggregate context: OpenRouter alone routed ~100T tokens/month (May 2026, 5x in 6 months); Google reported &gt;3.2 quadrillion tokens/month across products (I/O 2026); Meta burned ~70T/month (Feb 2026, SemiAnalysis).</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A27:G27"/>
+    <mergeCell ref="A21:G21"/>
+    <mergeCell ref="A22:G22"/>
+    <mergeCell ref="A26:G26"/>
+    <mergeCell ref="A24:G24"/>
+    <mergeCell ref="A25:G25"/>
+    <mergeCell ref="A23:G23"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B5:E19">
+    <cfRule type="dataBar" priority="1">
+      <dataBar showValue="1">
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="0070AD47"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -19568,7 +20400,29 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="B74:B74"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="74">
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Y axes are logarithmic. Gaps before a lineage's first launch are blank. Source: Quarterly Series sheet.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -19976,20 +20830,152 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>Ramp - AI token cost benchmarks (AI Index, Apr-Jun 2026)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Token Usage sheet anchors: $0.72/1M effective rate, median/average company spend, 1,001% usage growth Jan 2025-Apr 2026, PEPM benchmarks</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>https://ramp.com/blog/ai-token-cost-for-businesses</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>OpenAI - Enterprise Signals</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Token Usage sheet: frontier firms generate 8.3x output tokens per active user vs typical firms (Jun 2026)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>https://openai.com/signals/enterprise-data/</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>TechStartups - OpenRouter Series B (Deloitte 2026 study cited)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Token Usage sheet: 67% of enterprises consume &gt;1B tokens/month; OpenRouter ~100T tokens/month, 5x in 6 months</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>https://techstartups.com/2026/05/26/openrouter-raises-113m-as-ai-token-usage-surges-to-100-trillion-monthly/</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>VendorBenchmark - Enterprise GenAI cost benchmark 2026</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Token Usage sheet: enterprise LLM API spend $4-22 per employee/month; segment PEPM ranges</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>https://vendorbenchmark.com/guides/enterprise-genai-cost-benchmark-2026</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>SemiAnalysis - TokenBudgeting newsletter</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Token Usage sheet: Meta ~70T tokens/month (Feb 2026); enterprise spend percentiles</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>https://newsletter.semianalysis.com/p/tokenbudgeting-our-conversations</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Trending Topics EU - open-weight share of AI usage</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Aggregate token volumes: Google &gt;3.2 quadrillion tokens/month (I/O 2026), OpenAI API ~260T/month (Oct 2025)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>https://www.trendingtopics.eu/open-weight-models-from-china-are-capturing-a-growing-share-of-ai-usage/</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>Vendor announcements 2023-2025 (compiled)</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>Historical launch prices: GPT-4/Turbo/4o, Claude 2/3/4, Gemini 1.5-2.5, Grok 2-4, Llama 2-4, DeepSeek V2-V3.2, Kimi K2, GLM-4.5+</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>various (see notes column in Price History)</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>

</xml_diff>